<commit_message>
panier + historique de commande
</commit_message>
<xml_diff>
--- a/Fonctionnalités_Projet.xlsx
+++ b/Fonctionnalités_Projet.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58FBEF2D-D17F-4E11-B695-48E6E0F5C418}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66F17E95-9161-4306-9ECE-034BC719259E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="134">
   <si>
     <t xml:space="preserve">NOM ELEVE : </t>
   </si>
@@ -2961,12 +2961,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3257,18 +3257,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5" t="s">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="C2" s="3"/>
@@ -3303,7 +3303,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B8" s="6"/>
+      <c r="B8" s="5"/>
       <c r="C8" s="3" t="s">
         <v>9</v>
       </c>
@@ -3312,7 +3312,7 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B9" s="7"/>
+      <c r="B9" s="6"/>
       <c r="C9" s="3"/>
       <c r="D9" t="s">
         <v>20</v>
@@ -3330,7 +3330,7 @@
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B12" s="6"/>
+      <c r="B12" s="5"/>
       <c r="C12" s="3" t="s">
         <v>9</v>
       </c>
@@ -3339,7 +3339,7 @@
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B13" s="6"/>
+      <c r="B13" s="5"/>
       <c r="C13" s="3" t="s">
         <v>9</v>
       </c>
@@ -3348,7 +3348,7 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B14" s="6"/>
+      <c r="B14" s="5"/>
       <c r="C14" s="3" t="s">
         <v>9</v>
       </c>
@@ -3357,7 +3357,7 @@
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B15" s="6"/>
+      <c r="B15" s="5"/>
       <c r="C15" s="3" t="s">
         <v>9</v>
       </c>
@@ -3366,7 +3366,7 @@
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B16" s="8"/>
+      <c r="B16" s="7"/>
       <c r="C16" s="3" t="s">
         <v>11</v>
       </c>
@@ -3375,7 +3375,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B17" s="6"/>
+      <c r="B17" s="5"/>
       <c r="C17" s="3" t="s">
         <v>9</v>
       </c>
@@ -3395,7 +3395,7 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B20" s="6"/>
+      <c r="B20" s="5"/>
       <c r="C20" s="3" t="s">
         <v>9</v>
       </c>
@@ -3424,7 +3424,7 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B25" s="6"/>
+      <c r="B25" s="5"/>
       <c r="C25" s="3" t="s">
         <v>9</v>
       </c>
@@ -3433,25 +3433,37 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C26" s="3"/>
+      <c r="B26" s="5"/>
+      <c r="C26" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="D26" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C27" s="3"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="D27" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C28" s="3"/>
+      <c r="B28" s="5"/>
+      <c r="C28" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="D28" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C29" s="3"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="D29" t="s">
         <v>35</v>
       </c>
@@ -3468,19 +3480,28 @@
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C32" s="3"/>
+      <c r="B32" s="5"/>
+      <c r="C32" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="D32" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C33" s="3"/>
+      <c r="B33" s="5"/>
+      <c r="C33" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="D33" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C34" s="3"/>
+      <c r="B34" s="5"/>
+      <c r="C34" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="D34" t="s">
         <v>38</v>
       </c>
@@ -3638,7 +3659,7 @@
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B62" s="6"/>
+      <c r="B62" s="5"/>
       <c r="C62" s="3" t="s">
         <v>9</v>
       </c>
@@ -3647,7 +3668,7 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B63" s="6"/>
+      <c r="B63" s="5"/>
       <c r="C63" s="3" t="s">
         <v>9</v>
       </c>
@@ -3661,18 +3682,25 @@
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C65" s="3"/>
+      <c r="B65" s="5"/>
+      <c r="C65" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="D65" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C66" s="3"/>
+      <c r="B66" s="5"/>
+      <c r="C66" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="D66" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B67" s="6"/>
       <c r="C67" s="3"/>
       <c r="D67" t="s">
         <v>60</v>
@@ -4185,7 +4213,7 @@
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B159" s="6"/>
+      <c r="B159" s="5"/>
       <c r="C159" s="3" t="s">
         <v>9</v>
       </c>
@@ -4479,7 +4507,7 @@
       </c>
       <c r="B4">
         <f>COUNTIF(Feuil1!C8:'Feuil1'!C230,"X")</f>
-        <v>11</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
nouvelle page mode admin + rajout de vin + bdd pour les presta
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/Fonctionnalités_Projet.xlsx
+++ b/Fonctionnalités_Projet.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66F17E95-9161-4306-9ECE-034BC719259E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F47F166-ECCD-43DF-BEEB-7344FAA955E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="134">
   <si>
     <t xml:space="preserve">NOM ELEVE : </t>
   </si>
@@ -2951,7 +2951,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2966,6 +2966,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3527,42 +3530,51 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39" s="9">
+        <v>1</v>
+      </c>
       <c r="C39" s="3"/>
       <c r="D39" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A40" s="9"/>
       <c r="C40" s="3"/>
       <c r="D40" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" s="9"/>
       <c r="C41" s="3"/>
       <c r="D41" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A42" s="9"/>
       <c r="C42" s="3"/>
       <c r="D42" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A43" s="9"/>
       <c r="C43" s="3"/>
       <c r="D43" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A44" s="9"/>
       <c r="C44" s="3"/>
       <c r="D44" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A45" s="9"/>
       <c r="C45" s="3"/>
       <c r="D45" t="s">
         <v>54</v>
@@ -3707,13 +3719,19 @@
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C68" s="3"/>
+      <c r="B68" s="5"/>
+      <c r="C68" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="D68" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C69" s="3"/>
+      <c r="B69" s="5"/>
+      <c r="C69" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="D69" t="s">
         <v>62</v>
       </c>
@@ -3730,31 +3748,46 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C72" s="3"/>
+      <c r="B72" s="5"/>
+      <c r="C72" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="D72" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C73" s="3"/>
+      <c r="B73" s="5"/>
+      <c r="C73" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="D73" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C74" s="3"/>
+      <c r="B74" s="5"/>
+      <c r="C74" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="D74" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C75" s="3"/>
+      <c r="B75" s="5"/>
+      <c r="C75" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="D75" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C76" s="3"/>
+      <c r="B76" s="7"/>
+      <c r="C76" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="D76" t="s">
         <v>67</v>
       </c>
@@ -4478,9 +4511,10 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:H1"/>
+    <mergeCell ref="A39:A45"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -4489,25 +4523,29 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2646D6AF-1D80-493F-A7C9-967D3419C648}">
-  <dimension ref="A3:B4"/>
+  <dimension ref="A3:C4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>11</v>
       </c>
       <c r="B3">
         <f>COUNTIF(Feuil1!C7:'Feuil1'!C229,"P")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>9</v>
       </c>
       <c r="B4">
         <f>COUNTIF(Feuil1!C8:'Feuil1'!C230,"X")</f>
-        <v>20</v>
+        <v>26</v>
+      </c>
+      <c r="C4">
+        <f>B4*0.25+B3*0.125</f>
+        <v>6.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>